<commit_message>
Add List Conversation request type to data modeling workbook
Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Thoth data modeling.xlsx
+++ b/docs/Thoth data modeling.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="115" uniqueCount="35">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="125" uniqueCount="36">
   <si>
     <t>Conversations</t>
   </si>
@@ -101,6 +101,9 @@
   </si>
   <si>
     <t>Attachments[]</t>
+  </si>
+  <si>
+    <t>List Conversation request</t>
   </si>
   <si>
     <t>LLMMessageType</t>
@@ -761,19 +764,53 @@
       </c>
     </row>
     <row r="19">
+      <c r="A19" s="1" t="s">
+        <v>30</v>
+      </c>
       <c r="I19" s="5" t="s">
         <v>4</v>
       </c>
       <c r="J19" s="5" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="K19" s="5" t="s">
         <v>8</v>
       </c>
     </row>
+    <row r="20">
+      <c r="A20" s="4" t="s">
+        <v>3</v>
+      </c>
+      <c r="B20" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="B21" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>8</v>
+      </c>
+    </row>
     <row r="22">
+      <c r="A22" s="5" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>8</v>
+      </c>
       <c r="I22" s="3" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
     <row r="23">
@@ -792,7 +829,7 @@
         <v>20</v>
       </c>
       <c r="J24" s="5" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="K24" s="5" t="s">
         <v>8</v>
@@ -803,7 +840,7 @@
         <v>14</v>
       </c>
       <c r="J25" s="5" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="K25" s="5" t="s">
         <v>8</v>
@@ -811,17 +848,17 @@
     </row>
     <row r="26">
       <c r="I26" s="5" t="s">
+        <v>35</v>
+      </c>
+      <c r="J26" s="5" t="s">
         <v>34</v>
       </c>
-      <c r="J26" s="5" t="s">
-        <v>33</v>
-      </c>
       <c r="K26" s="5" t="s">
         <v>8</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="8">
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="E3:G3"/>
     <mergeCell ref="I3:K3"/>
@@ -829,6 +866,7 @@
     <mergeCell ref="I22:K22"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A15:C15"/>
+    <mergeCell ref="A19:C19"/>
   </mergeCells>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>